<commit_message>
CORREÇÕES E IMPLEMNETAÇÃO D EPLANO PREMIUM
</commit_message>
<xml_diff>
--- a/relatorios/financas_2026-05.xlsx
+++ b/relatorios/financas_2026-05.xlsx
@@ -8,16 +8,17 @@
     <sheet sheetId="2" name="💰 Ganhos" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="💸 Gastos" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="📋 Contas Fixas" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="🏷️ Categorias" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="📈 Comparação" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="📐 Médias" state="visible" r:id="rId10"/>
+    <sheet sheetId="5" name="✅❌ Adim. &amp; Inadim." state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="🏷️ Categorias" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="📈 Comparação" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="📐 Médias" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="73">
   <si>
     <t>RESUMO FINANCEIRO — MAIO 2026</t>
   </si>
@@ -91,13 +92,22 @@
     <t>TOTAL</t>
   </si>
   <si>
+    <t>2026-05-11</t>
+  </si>
+  <si>
+    <t>mercado</t>
+  </si>
+  <si>
+    <t>Alimentação</t>
+  </si>
+  <si>
     <t>Vencimento (Dia)</t>
   </si>
   <si>
     <t>Ativa?</t>
   </si>
   <si>
-    <t>sicred</t>
+    <t>sicredi</t>
   </si>
   <si>
     <t>Cartão de Crédito</t>
@@ -139,6 +149,45 @@
     <t>TOTAL MENSAL</t>
   </si>
   <si>
+    <t>ADIMPLÊNCIA &amp; INADIMPLÊNCIA — MAIO 2026</t>
+  </si>
+  <si>
+    <t>Métrica</t>
+  </si>
+  <si>
+    <t>Total de contas fixas ativas</t>
+  </si>
+  <si>
+    <t>✓ Contas pagas</t>
+  </si>
+  <si>
+    <t>✓ Valor pago</t>
+  </si>
+  <si>
+    <t>✓ Adimplência (%)</t>
+  </si>
+  <si>
+    <t>⚠ Contas vencidas</t>
+  </si>
+  <si>
+    <t>⚠ Valor vencido</t>
+  </si>
+  <si>
+    <t>⚠ Inadimplência (%)</t>
+  </si>
+  <si>
+    <t>CONTAS PAGAS NO MÊS</t>
+  </si>
+  <si>
+    <t>CONTAS NÃO PAGAS NO MÊS</t>
+  </si>
+  <si>
+    <t>Vencida?</t>
+  </si>
+  <si>
+    <t>Não</t>
+  </si>
+  <si>
     <t>GANHOS POR CATEGORIA</t>
   </si>
   <si>
@@ -155,9 +204,6 @@
   </si>
   <si>
     <t>COMPARAÇÃO: ABRIL 2026 → MAIO 2026</t>
-  </si>
-  <si>
-    <t>Métrica</t>
   </si>
   <si>
     <t>abril 2026</t>
@@ -240,7 +286,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -284,6 +330,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="70AD47"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="C6EFCE"/>
       </patternFill>
     </fill>
@@ -320,7 +376,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -373,6 +429,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -380,46 +439,64 @@
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -816,7 +893,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="6">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -824,7 +901,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="8">
-        <v>3715</v>
+        <v>3770</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -832,7 +909,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="6">
-        <v>3715</v>
+        <v>3870</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -840,7 +917,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="10">
-        <v>-755</v>
+        <v>-2910</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -848,7 +925,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="11">
-        <v>-25.506756756756754</v>
+        <v>-98.3108108108108</v>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -976,7 +1053,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -997,6 +1074,34 @@
       </c>
       <c r="D1" s="2" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="6">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="19">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1026,98 +1131,98 @@
         <v>16</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>17</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" s="20" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" s="21">
-        <v>670</v>
-      </c>
-      <c r="E2" s="20" t="s">
+      <c r="A2" s="21" t="s">
         <v>29</v>
       </c>
+      <c r="B2" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="22">
+        <v>673</v>
+      </c>
+      <c r="E2" s="21" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="24">
+        <v>120</v>
+      </c>
+      <c r="E3" s="23" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="D3" s="23">
-        <v>120</v>
-      </c>
-      <c r="E3" s="22" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="20" t="s">
+      <c r="C4" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" s="22">
+        <v>2852</v>
+      </c>
+      <c r="E4" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="D4" s="21">
-        <v>2800</v>
-      </c>
-      <c r="E4" s="20" t="s">
-        <v>29</v>
-      </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="22" t="s">
-        <v>34</v>
-      </c>
-      <c r="B5" s="22" t="s">
-        <v>35</v>
-      </c>
-      <c r="C5" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="D5" s="23">
+      <c r="A5" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="24">
         <v>40</v>
       </c>
-      <c r="E5" s="22" t="s">
-        <v>29</v>
+      <c r="E5" s="23" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="B6" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="C6" s="20" t="s">
-        <v>38</v>
-      </c>
-      <c r="D6" s="21">
+      <c r="A6" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" s="22">
         <v>85</v>
       </c>
-      <c r="E6" s="20" t="s">
-        <v>29</v>
+      <c r="E6" s="21" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -1125,13 +1230,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C7" s="17" t="s">
         <v>3</v>
       </c>
       <c r="D7" s="19">
-        <v>3715</v>
+        <v>3770</v>
       </c>
       <c r="E7" s="17" t="s">
         <v>3</v>
@@ -1145,7 +1250,240 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="35" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="25" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="27">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="28" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="4">
+        <v>3645</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="28" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="30">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="28" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="31" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12" s="31"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="31"/>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14" s="4">
+        <v>673</v>
+      </c>
+      <c r="E14" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="16">
+        <v>120</v>
+      </c>
+      <c r="E15" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="4">
+        <v>2852</v>
+      </c>
+      <c r="E16" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" s="32"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="E19" s="25" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="33" t="s">
+        <v>37</v>
+      </c>
+      <c r="B20" s="33" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" s="33" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" s="8">
+        <v>40</v>
+      </c>
+      <c r="E20" s="33" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D21" s="16">
+        <v>85</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A18:E18"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1156,28 +1494,28 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="B2" s="24" t="s">
+      <c r="A2" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="24" t="s">
-        <v>42</v>
+      <c r="D2" s="25" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="25">
+      <c r="A3" s="29">
         <v>1</v>
       </c>
       <c r="B3" s="14" t="s">
@@ -1186,12 +1524,12 @@
       <c r="C3" s="4">
         <v>2760</v>
       </c>
-      <c r="D3" s="26">
+      <c r="D3" s="30">
         <v>93.24324324324324</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="27">
+      <c r="A4" s="34">
         <v>2</v>
       </c>
       <c r="B4" s="15" t="s">
@@ -1200,122 +1538,136 @@
       <c r="C4" s="16">
         <v>200</v>
       </c>
-      <c r="D4" s="28">
+      <c r="D4" s="35">
         <v>6.756756756756757</v>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="B7" s="24" t="s">
+      <c r="A7" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="B7" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="C7" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="24" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="B10" s="24" t="s">
+      <c r="D7" s="25" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="36">
+        <v>1</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="6">
+        <v>100</v>
+      </c>
+      <c r="D8" s="37">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="C11" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="24" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="29">
+      <c r="D11" s="25" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="38">
         <v>1</v>
       </c>
-      <c r="B11" s="30" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="8">
-        <v>3470</v>
-      </c>
-      <c r="D11" s="31">
-        <v>93.40511440107672</v>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="27">
+      <c r="B12" s="33" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="8">
+        <v>3525</v>
+      </c>
+      <c r="D12" s="39">
+        <v>93.50132625994695</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="34">
         <v>2</v>
       </c>
-      <c r="B12" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12" s="16">
+      <c r="B13" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13" s="16">
         <v>120</v>
       </c>
-      <c r="D12" s="28">
-        <v>3.2301480484522207</v>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="29">
+      <c r="D13" s="35">
+        <v>3.183023872679045</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="38">
         <v>3</v>
       </c>
-      <c r="B13" s="30" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" s="8">
+      <c r="B14" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="8">
         <v>85</v>
       </c>
-      <c r="D13" s="31">
-        <v>2.2880215343203227</v>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="27">
+      <c r="D14" s="39">
+        <v>2.2546419098143233</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="34">
         <v>4</v>
       </c>
-      <c r="B14" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="C14" s="16">
+      <c r="B15" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="16">
         <v>40</v>
       </c>
-      <c r="D14" s="28">
-        <v>1.0767160161507403</v>
+      <c r="D15" s="35">
+        <v>1.0610079575596816</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A10:D10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1328,7 +1680,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1336,25 +1688,25 @@
       <c r="E1" s="2"/>
     </row>
     <row r="2" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
-        <v>46</v>
-      </c>
-      <c r="B2" s="24" t="s">
-        <v>47</v>
-      </c>
-      <c r="C2" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="D2" s="24" t="s">
-        <v>49</v>
-      </c>
-      <c r="E2" s="24" t="s">
-        <v>50</v>
+      <c r="A2" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="32" t="s">
-        <v>51</v>
+      <c r="A3" s="40" t="s">
+        <v>66</v>
       </c>
       <c r="B3" s="16">
         <v>0</v>
@@ -1362,79 +1714,79 @@
       <c r="C3" s="16">
         <v>2960</v>
       </c>
-      <c r="D3" s="33">
+      <c r="D3" s="41">
         <v>2960</v>
       </c>
-      <c r="E3" s="34">
+      <c r="E3" s="42">
         <v>100</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="36">
+      <c r="B4" s="44">
         <v>0</v>
       </c>
-      <c r="C4" s="36">
+      <c r="C4" s="44">
+        <v>100</v>
+      </c>
+      <c r="D4" s="10">
+        <v>100</v>
+      </c>
+      <c r="E4" s="11">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="40" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="16">
         <v>0</v>
       </c>
-      <c r="D4" s="36">
+      <c r="C5" s="16">
+        <v>3770</v>
+      </c>
+      <c r="D5" s="10">
+        <v>3770</v>
+      </c>
+      <c r="E5" s="45" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="43" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" s="44">
         <v>0</v>
       </c>
-      <c r="E4" s="37">
+      <c r="C6" s="44">
+        <v>3870</v>
+      </c>
+      <c r="D6" s="10">
+        <v>3870</v>
+      </c>
+      <c r="E6" s="11">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="40" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" s="16">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="32" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="16">
-        <v>3715</v>
-      </c>
-      <c r="C5" s="16">
-        <v>3715</v>
-      </c>
-      <c r="D5" s="16">
-        <v>0</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="35" t="s">
-        <v>53</v>
-      </c>
-      <c r="B6" s="36">
-        <v>3715</v>
-      </c>
-      <c r="C6" s="36">
-        <v>3715</v>
-      </c>
-      <c r="D6" s="36">
-        <v>0</v>
-      </c>
-      <c r="E6" s="37">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="32" t="s">
-        <v>54</v>
-      </c>
-      <c r="B7" s="16">
-        <v>-3715</v>
-      </c>
       <c r="C7" s="16">
-        <v>-755</v>
-      </c>
-      <c r="D7" s="33">
-        <v>2960</v>
-      </c>
-      <c r="E7" s="34">
-        <v>79.67698519515478</v>
+        <v>-2910</v>
+      </c>
+      <c r="D7" s="10">
+        <v>-2910</v>
+      </c>
+      <c r="E7" s="11">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1446,7 +1798,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1457,64 +1809,64 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="B1" s="2"/>
     </row>
     <row r="2" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
-        <v>46</v>
-      </c>
-      <c r="B2" s="24" t="s">
-        <v>56</v>
+      <c r="A2" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="38" t="s">
-        <v>51</v>
+      <c r="A3" s="28" t="s">
+        <v>66</v>
       </c>
       <c r="B3" s="4">
         <v>2960</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="39" t="s">
+      <c r="A4" s="46" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="6">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="40" t="s">
+      <c r="A5" s="47" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="8">
-        <v>3715</v>
+        <v>3770</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="39" t="s">
+      <c r="A6" s="46" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="6">
-        <v>3715</v>
+        <v>3870</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="41" t="s">
-        <v>54</v>
+      <c r="A7" s="48" t="s">
+        <v>69</v>
       </c>
       <c r="B7" s="10">
-        <v>-755</v>
+        <v>-2910</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="32" t="s">
-        <v>57</v>
-      </c>
-      <c r="B8" s="28">
-        <v>-25.506756756756754</v>
+      <c r="A8" s="40" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" s="35">
+        <v>-98.3108108108108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>